<commit_message>
security-tools-mapping-navigator: fix template record_id and CIS-3 tool mapping
- Tool Inventory: add record_id as col A with auto-fill formula (="MAP-"&ROW()-3)
- Instructions: record_id description updated from "leave blank" to "auto-filled in template"
- Instructions CIS-3 example tools: remove Proofpoint/Mimecast (email tools, belong in CIS-9)
  and replace with Microsoft Purview, Varonis, Symantec DLP, Forcepoint

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
+++ b/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -119,8 +119,17 @@
       <i val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -196,6 +205,26 @@
         <fgColor rgb="00f0f8f9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000a3541"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff9c4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00fff6e5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00e8f5e9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -223,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -328,6 +357,16 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -775,7 +814,7 @@
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
-          <t>Not in the template — the app auto-generates a unique record ID for every row on upload.</t>
+          <t>Auto-filled in the template using a formula. You can also leave it empty — the app assigns IDs on upload.</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1326,7 @@
       </c>
       <c r="D41" s="25" t="inlineStr">
         <is>
-          <t>Proofpoint, Mimecast, Microsoft Purview, Varonis</t>
+          <t>Microsoft Purview, Varonis, Symantec DLP, Forcepoint</t>
         </is>
       </c>
     </row>
@@ -1672,10 +1711,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -1689,506 +1728,540 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>record_id</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>tool_name *</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>vendor *</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>product *</t>
         </is>
       </c>
-      <c r="D1" s="17" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>control_domain *</t>
         </is>
       </c>
-      <c r="E1" s="17" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>control_objective *</t>
         </is>
       </c>
-      <c r="F1" s="16" t="inlineStr">
+      <c r="G1" s="16" t="inlineStr">
         <is>
           <t>current_control_id</t>
         </is>
       </c>
-      <c r="G1" s="16" t="inlineStr">
+      <c r="H1" s="16" t="inlineStr">
         <is>
           <t>framework_alignment</t>
         </is>
       </c>
-      <c r="H1" s="16" t="inlineStr">
+      <c r="I1" s="16" t="inlineStr">
         <is>
           <t>coverage_level</t>
         </is>
       </c>
-      <c r="I1" s="16" t="inlineStr">
+      <c r="J1" s="16" t="inlineStr">
         <is>
           <t>operational_status</t>
         </is>
       </c>
-      <c r="J1" s="16" t="inlineStr">
+      <c r="K1" s="16" t="inlineStr">
         <is>
           <t>annual_cost_usd</t>
         </is>
       </c>
-      <c r="K1" s="16" t="inlineStr">
+      <c r="L1" s="16" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>auto-generated</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>e.g. Identity Access Platform  [REQUIRED]</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>e.g. Microsoft  [REQUIRED]</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>e.g. Entra ID P2  [REQUIRED]</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="E2" s="18" t="inlineStr">
         <is>
           <t>Identity / Endpoint / Network / Data / Cloud / AppSec / SOC  [REQUIRED]</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="F2" s="18" t="inlineStr">
         <is>
           <t>Describe what this tool protects or detects — be specific  [REQUIRED]</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>e.g. PR.AA  or  CIS-5  (see reference tables in Instructions)</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0 / CIS-v8.1 / NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="I2" s="18" t="inlineStr">
         <is>
           <t>Fully Covered / Partially Covered / Minimally Covered / Not Covered</t>
         </is>
       </c>
-      <c r="I2" s="18" t="inlineStr">
+      <c r="J2" s="18" t="inlineStr">
         <is>
           <t>Active / Planned / Inactive</t>
         </is>
       </c>
-      <c r="J2" s="18" t="inlineStr">
+      <c r="K2" s="18" t="inlineStr">
         <is>
           <t>Annual spend in USD (used for redundancy savings estimate)</t>
         </is>
       </c>
-      <c r="K2" s="18" t="inlineStr">
+      <c r="L2" s="18" t="inlineStr">
         <is>
           <t>Any additional context — scope, known gaps, integrations</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Delete the seven example rows below (rows 4–10) before uploading your data.</t>
-        </is>
-      </c>
+      <c r="A3" s="43" t="n"/>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>Identity Access Platform</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Entra ID P2</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Identity and privileged access governance for all enterprise user accounts</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="G4" s="20" t="inlineStr">
         <is>
           <t>PR.AA</t>
         </is>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Partially Covered</t>
         </is>
       </c>
-      <c r="I4" s="20" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J4" s="20" t="n">
+      <c r="K4" s="20" t="n">
         <v>250000</v>
       </c>
-      <c r="K4" s="20" t="inlineStr">
+      <c r="L4" s="20" t="inlineStr">
         <is>
           <t>Legacy MFA methods still enabled on 8% of accounts</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Endpoint Detection and Response</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>CrowdStrike</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>Falcon Insight XDR</t>
         </is>
       </c>
-      <c r="D5" s="20" t="inlineStr">
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="E5" s="20" t="inlineStr">
+      <c r="F5" s="20" t="inlineStr">
         <is>
           <t>Endpoint detection and response for workstations and servers</t>
         </is>
       </c>
-      <c r="F5" s="20" t="inlineStr">
+      <c r="G5" s="20" t="inlineStr">
         <is>
           <t>PR.PS</t>
         </is>
       </c>
-      <c r="G5" s="20" t="inlineStr">
+      <c r="H5" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H5" s="20" t="inlineStr">
+      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>Fully Covered</t>
         </is>
       </c>
-      <c r="I5" s="20" t="inlineStr">
+      <c r="J5" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="K5" s="20" t="n">
         <v>380000</v>
       </c>
-      <c r="K5" s="20" t="inlineStr">
+      <c r="L5" s="20" t="inlineStr">
         <is>
           <t>Deployed to all managed endpoints; unmanaged devices not covered</t>
         </is>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B6" s="20" t="inlineStr">
         <is>
           <t>Next-Generation Firewall</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>Palo Alto Networks</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="D6" s="20" t="inlineStr">
         <is>
           <t>PA-Series NGFW</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>Network</t>
         </is>
       </c>
-      <c r="E6" s="20" t="inlineStr">
+      <c r="F6" s="20" t="inlineStr">
         <is>
           <t>Network boundary and segmentation controls for perimeter and east-west traffic</t>
         </is>
       </c>
-      <c r="F6" s="20" t="inlineStr">
+      <c r="G6" s="20" t="inlineStr">
         <is>
           <t>PR.IR</t>
         </is>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="H6" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
+      <c r="I6" s="20" t="inlineStr">
         <is>
           <t>Fully Covered</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr">
+      <c r="J6" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="K6" s="20" t="n">
         <v>210000</v>
       </c>
-      <c r="K6" s="20" t="inlineStr">
+      <c r="L6" s="20" t="inlineStr">
         <is>
           <t>HA pair at HQ; branch offices use older ASA</t>
         </is>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>Email Security Gateway</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Proofpoint</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>Essentials</t>
         </is>
       </c>
-      <c r="D7" s="20" t="inlineStr">
+      <c r="E7" s="20" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr">
+      <c r="F7" s="20" t="inlineStr">
         <is>
           <t>Data security and email threat prevention for inbound and outbound communications</t>
         </is>
       </c>
-      <c r="F7" s="20" t="inlineStr">
+      <c r="G7" s="20" t="inlineStr">
         <is>
           <t>PR.DS</t>
         </is>
       </c>
-      <c r="G7" s="20" t="inlineStr">
+      <c r="H7" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H7" s="20" t="inlineStr">
+      <c r="I7" s="20" t="inlineStr">
         <is>
           <t>Partially Covered</t>
         </is>
       </c>
-      <c r="I7" s="20" t="inlineStr">
+      <c r="J7" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="K7" s="20" t="n">
         <v>95000</v>
       </c>
-      <c r="K7" s="20" t="inlineStr">
+      <c r="L7" s="20" t="inlineStr">
         <is>
           <t>DLP rules not fully configured; attachment sandboxing active</t>
         </is>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B8" s="20" t="inlineStr">
         <is>
           <t>Cloud Security Posture Management</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="C8" s="20" t="inlineStr">
         <is>
           <t>Wiz</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="D8" s="20" t="inlineStr">
         <is>
           <t>CNAPP</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>Cloud</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr">
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>Cloud security posture and workload protection for cloud-hosted infrastructure and applications</t>
         </is>
       </c>
-      <c r="F8" s="20" t="inlineStr">
+      <c r="G8" s="20" t="inlineStr">
         <is>
           <t>CIS-4</t>
         </is>
       </c>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H8" s="20" t="inlineStr">
+      <c r="I8" s="20" t="inlineStr">
         <is>
           <t>Partially Covered</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr">
+      <c r="J8" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="K8" s="20" t="n">
         <v>220000</v>
       </c>
-      <c r="K8" s="20" t="inlineStr">
+      <c r="L8" s="20" t="inlineStr">
         <is>
           <t>Multi-cloud coverage; IaC scanning not yet enabled</t>
         </is>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Web Application Firewall</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Imperva</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Cloud WAF</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>AppSec</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr">
         <is>
           <t>Web application and API protection against OWASP Top 10 and injection attacks</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr">
+      <c r="G9" s="20" t="inlineStr">
         <is>
           <t>CIS-16</t>
         </is>
       </c>
-      <c r="G9" s="20" t="inlineStr">
+      <c r="H9" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H9" s="20" t="inlineStr">
+      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>Minimally Covered</t>
         </is>
       </c>
-      <c r="I9" s="20" t="inlineStr">
+      <c r="J9" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J9" s="20" t="n">
+      <c r="K9" s="20" t="n">
         <v>85000</v>
       </c>
-      <c r="K9" s="20" t="inlineStr">
+      <c r="L9" s="20" t="inlineStr">
         <is>
           <t>Runtime protection active; DAST integration pending</t>
         </is>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="44">
+        <f>"MAP-"&amp;(ROW()-3)</f>
+        <v/>
+      </c>
+      <c r="B10" s="20" t="inlineStr">
         <is>
           <t>Security Information and Event Management</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="D10" s="20" t="inlineStr">
         <is>
           <t>Microsoft Sentinel</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>SOC</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr">
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>Centralized security monitoring detection and response for hybrid environment</t>
         </is>
       </c>
-      <c r="F10" s="20" t="inlineStr">
+      <c r="G10" s="20" t="inlineStr">
         <is>
           <t>DE.CM</t>
         </is>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>NIST-CSF-2.0;CIS-v8.1</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
+      <c r="I10" s="20" t="inlineStr">
         <is>
           <t>Partially Covered</t>
         </is>
       </c>
-      <c r="I10" s="20" t="inlineStr">
+      <c r="J10" s="20" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="K10" s="20" t="n">
         <v>175000</v>
       </c>
-      <c r="K10" s="20" t="inlineStr">
+      <c r="L10" s="20" t="inlineStr">
         <is>
           <t>Log coverage gaps in OT and legacy systems</t>
         </is>
@@ -2196,7 +2269,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A3:L3"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
security-tools-mapping-navigator: fix Excel template dropdowns and Instructions cross-references
- Remove stale data validations (were stuck on wrong columns after record_id insert)
- Re-apply dropdowns on correct columns: E=control_domain, H=framework_alignment,
  I=coverage_level, J=operational_status; product and current_control_id no longer have dropdowns
- Instructions column reference: append "See valid values below." to descriptions
  for control_domain, framework_alignment, coverage_level, operational_status

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
+++ b/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
@@ -902,7 +902,7 @@
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>Must be one of: Identity | Endpoint | Network | Data | Cloud | AppSec | SOC</t>
+          <t>Must be one of: Identity | Endpoint | Network | Data | Cloud | AppSec | SOC  —  See valid values below.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="D15" s="26" t="inlineStr">
         <is>
-          <t>NIST-CSF-2.0  |  CIS-v8.1  |  NIST-CSF-2.0;CIS-v8.1</t>
+          <t>NIST-CSF-2.0  |  CIS-v8.1  |  NIST-CSF-2.0;CIS-v8.1  —  See valid values below.</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
-          <t>Fully Covered / Partially Covered / Minimally Covered / Not Covered — captures both coverage completeness and utilisation level.</t>
+          <t>Fully Covered / Partially Covered / Minimally Covered / Not Covered — captures both coverage completeness and utilisation level.  —  See valid values below.</t>
         </is>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="D17" s="26" t="inlineStr">
         <is>
-          <t>Active | Planned | Inactive.  Inactive = potential shelfware.</t>
+          <t>Active | Planned | Inactive.  Inactive = potential shelfware.  —  See valid values below.</t>
         </is>
       </c>
     </row>
@@ -2272,16 +2272,16 @@
     <mergeCell ref="A3:L3"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="D4:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E4:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Identity,Endpoint,Network,Data,Cloud,AppSec,SOC"</formula1>
     </dataValidation>
-    <dataValidation sqref="G4:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H4:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NIST-CSF-2.0,CIS-v8.1,NIST-CSF-2.0;CIS-v8.1"</formula1>
     </dataValidation>
-    <dataValidation sqref="H4:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="I4:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Fully Covered,Partially Covered,Minimally Covered,Not Covered"</formula1>
     </dataValidation>
-    <dataValidation sqref="I4:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J4:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Active,Planned,Inactive"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
security-tools-mapping-navigator: fix vendor/product Required vs Recommended mismatch
Tool Inventory headers and hint row marked vendor and product as Required (*
and [REQUIRED]) but Instructions correctly said Recommended. Fixed to match:
- Row 1: 'vendor *' -> 'vendor', 'product *' -> 'product'
- Row 2: [REQUIRED] -> [RECOMMENDED] for both columns

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
+++ b/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
@@ -1740,12 +1740,12 @@
       </c>
       <c r="C1" s="17" t="inlineStr">
         <is>
-          <t>vendor *</t>
+          <t>vendor</t>
         </is>
       </c>
       <c r="D1" s="17" t="inlineStr">
         <is>
-          <t>product *</t>
+          <t>product</t>
         </is>
       </c>
       <c r="E1" s="17" t="inlineStr">
@@ -1802,12 +1802,12 @@
       </c>
       <c r="C2" s="18" t="inlineStr">
         <is>
-          <t>e.g. Microsoft  [REQUIRED]</t>
+          <t>e.g. Microsoft  [RECOMMENDED]</t>
         </is>
       </c>
       <c r="D2" s="18" t="inlineStr">
         <is>
-          <t>e.g. Entra ID P2  [REQUIRED]</t>
+          <t>e.g. Entra ID P2  [RECOMMENDED]</t>
         </is>
       </c>
       <c r="E2" s="18" t="inlineStr">

</xml_diff>

<commit_message>
security-tools-mapping-navigator: fix 5 content issues in Excel template
1. Tool Inventory row 3: restore lost warning note (was cleared by insert_cols)
2. Instructions PR.PS examples: add Wiz and Prisma Cloud — PR.PS covers cloud
   workloads not just endpoint tools
3. Instructions CIS-4 examples: replace Tenable (vuln scanner) with Microsoft
   Intune and AWS Config (actual config management tools)
4. Instructions Tips: add Data domain GOOD example (was the only domain missing)
5. Instructions coverage_level description: remove awkward double em-dash

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
+++ b/projects/security-tools-mapping-navigator/Security_Tools_Mapping_Template.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -127,6 +127,11 @@
     <font>
       <color rgb="00555555"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008a5600"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="18">
@@ -252,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -366,6 +371,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -733,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -990,7 +998,7 @@
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
-          <t>Fully Covered / Partially Covered / Minimally Covered / Not Covered — captures both coverage completeness and utilisation level.  —  See valid values below.</t>
+          <t>Fully Covered / Partially Covered / Minimally Covered / Not Covered. Captures both coverage completeness and utilisation level. See valid values below.</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1195,7 @@
       </c>
       <c r="D32" s="26" t="inlineStr">
         <is>
-          <t>CrowdStrike Falcon, SentinelOne, Defender for Endpoint</t>
+          <t>CrowdStrike Falcon, SentinelOne, Defender for Endpoint, Wiz, Prisma Cloud</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1356,7 @@
       </c>
       <c r="D42" s="26" t="inlineStr">
         <is>
-          <t>Wiz, Prisma Cloud, Defender for Cloud, Tenable</t>
+          <t>Wiz, Prisma Cloud, Defender for Cloud, Microsoft Intune, AWS Config</t>
         </is>
       </c>
     </row>
@@ -1652,36 +1660,48 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="39" t="inlineStr">
+      <c r="A62" s="37" t="inlineStr">
+        <is>
+          <t>GOOD</t>
+        </is>
+      </c>
+      <c r="B62" s="28" t="inlineStr">
+        <is>
+          <t>Email and data loss prevention covering sensitive data in motion and at rest</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="39" t="inlineStr">
         <is>
           <t>AVOID</t>
         </is>
       </c>
-      <c r="B62" s="32" t="inlineStr">
+      <c r="B63" s="32" t="inlineStr">
         <is>
           <t>Security tool         ← too vague, produces weak gap analysis</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="40" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="40" t="inlineStr">
         <is>
           <t>AVOID</t>
         </is>
       </c>
-      <c r="B63" s="34" t="inlineStr">
+      <c r="B64" s="34" t="inlineStr">
         <is>
           <t>Firewall              ← say what it controls or detects</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="39" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="39" t="inlineStr">
         <is>
           <t>AVOID</t>
         </is>
       </c>
-      <c r="B64" s="32" t="inlineStr">
+      <c r="B65" s="32" t="inlineStr">
         <is>
           <t>Monitoring            ← say what is monitored and why</t>
         </is>
@@ -1852,7 +1872,11 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="43" t="n"/>
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⚠  Delete the seven example rows below (rows 4–10) before uploading your data.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="44">

</xml_diff>